<commit_message>
Harden Phase-0 golden net: honest MC, tolerant OR, associative coverage.
Resample degenerate Monte Carlo draws instead of scoring chi2=0; lock homogeneous OR with approx; add nuclear associativa fixture sentence; record near wall-clock baseline for the Phase-1 ±20% budget.

Co-authored-by: Cursor <cursoragent@cursor.com>
</commit_message>
<xml_diff>
--- a/tests/fixtures/matriz_miniatura.xlsx
+++ b/tests/fixtures/matriz_miniatura.xlsx
@@ -697,11 +697,11 @@
       </c>
       <c r="O8" t="inlineStr">
         <is>
-          <t>the guitar textures combined with the lyrics of the singer created a dense surface</t>
+          <t>the combination of textures with the lyrics was striking in the final refrain of the song</t>
         </is>
       </c>
       <c r="P8" t="n">
-        <v>14</v>
+        <v>16</v>
       </c>
     </row>
     <row r="9">

</xml_diff>

<commit_message>
Fix MC p-value honesty, local perf gate, and restore incidental assoc fixture.
Skip degenerate MC draws and fall back to Fisher when validas are low; assert agreement with Fisher; mark wall-clock budget local_perf/CI-skip; keep both incidental and nuclear associative rows; resolve default dominios.tsv at project root.

Co-authored-by: Cursor <cursoragent@cursor.com>
</commit_message>
<xml_diff>
--- a/tests/fixtures/matriz_miniatura.xlsx
+++ b/tests/fixtures/matriz_miniatura.xlsx
@@ -413,7 +413,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:P27"/>
+  <dimension ref="A1:P28"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -697,11 +697,11 @@
       </c>
       <c r="O8" t="inlineStr">
         <is>
-          <t>the combination of textures with the lyrics was striking in the final refrain of the song</t>
+          <t>the guitar textures combined with the lyrics of the singer created a dense surface</t>
         </is>
       </c>
       <c r="P8" t="n">
-        <v>16</v>
+        <v>14</v>
       </c>
     </row>
     <row r="9">
@@ -712,7 +712,7 @@
       <c r="E9" t="inlineStr"/>
       <c r="F9" t="inlineStr">
         <is>
-          <t>texture</t>
+          <t>textures</t>
         </is>
       </c>
       <c r="G9" t="inlineStr"/>
@@ -722,7 +722,7 @@
       <c r="K9" t="inlineStr"/>
       <c r="L9" t="inlineStr">
         <is>
-          <t>E:\todos os textos\(2008)_Choir.pdf</t>
+          <t>E:\todos os textos\(2005)_Song_Assoc.pdf</t>
         </is>
       </c>
       <c r="M9" t="inlineStr"/>
@@ -733,11 +733,11 @@
       </c>
       <c r="O9" t="inlineStr">
         <is>
-          <t>the voices are combined into a homophonic texture of unusual clarity and warmth</t>
+          <t>the combination of textures with the lyrics was striking in the final refrain of the song</t>
         </is>
       </c>
       <c r="P9" t="n">
-        <v>13</v>
+        <v>16</v>
       </c>
     </row>
     <row r="10">
@@ -758,7 +758,7 @@
       <c r="K10" t="inlineStr"/>
       <c r="L10" t="inlineStr">
         <is>
-          <t>E:\todos os textos\(1960)_Medida_Complexity.pdf</t>
+          <t>E:\todos os textos\(2008)_Choir.pdf</t>
         </is>
       </c>
       <c r="M10" t="inlineStr"/>
@@ -769,11 +769,11 @@
       </c>
       <c r="O10" t="inlineStr">
         <is>
-          <t>clock which measures duration with which to measure the degree of textural complexity irvine asks the question about form</t>
+          <t>the voices are combined into a homophonic texture of unusual clarity and warmth</t>
         </is>
       </c>
       <c r="P10" t="n">
-        <v>19</v>
+        <v>13</v>
       </c>
     </row>
     <row r="11">
@@ -794,7 +794,7 @@
       <c r="K11" t="inlineStr"/>
       <c r="L11" t="inlineStr">
         <is>
-          <t>E:\todos os textos\Copia__ab12cd34.pdf</t>
+          <t>E:\todos os textos\(1960)_Medida_Complexity.pdf</t>
         </is>
       </c>
       <c r="M11" t="inlineStr"/>
@@ -805,11 +805,11 @@
       </c>
       <c r="O11" t="inlineStr">
         <is>
-          <t>ck which measures duration with which to measure the degree of textural complexity</t>
+          <t>clock which measures duration with which to measure the degree of textural complexity irvine asks the question about form</t>
         </is>
       </c>
       <c r="P11" t="n">
-        <v>13</v>
+        <v>19</v>
       </c>
     </row>
     <row r="12">
@@ -830,7 +830,7 @@
       <c r="K12" t="inlineStr"/>
       <c r="L12" t="inlineStr">
         <is>
-          <t>E:\todos os textos\(1955)_Homogeny.pdf</t>
+          <t>E:\todos os textos\Copia__ab12cd34.pdf</t>
         </is>
       </c>
       <c r="M12" t="inlineStr"/>
@@ -841,11 +841,11 @@
       </c>
       <c r="O12" t="inlineStr">
         <is>
-          <t>extent to which a homogeneous texture a texture in which all the parts share the same musical material and are</t>
+          <t>ck which measures duration with which to measure the degree of textural complexity</t>
         </is>
       </c>
       <c r="P12" t="n">
-        <v>20</v>
+        <v>13</v>
       </c>
     </row>
     <row r="13">
@@ -877,11 +877,11 @@
       </c>
       <c r="O13" t="inlineStr">
         <is>
-          <t>aping of a modem language extent to which a homogeneous texture a texture in which all the parts share the same</t>
+          <t>extent to which a homogeneous texture a texture in which all the parts share the same musical material and are</t>
         </is>
       </c>
       <c r="P13" t="n">
-        <v>21</v>
+        <v>20</v>
       </c>
     </row>
     <row r="14">
@@ -892,7 +892,7 @@
       <c r="E14" t="inlineStr"/>
       <c r="F14" t="inlineStr">
         <is>
-          <t>textures</t>
+          <t>texture</t>
         </is>
       </c>
       <c r="G14" t="inlineStr"/>
@@ -902,7 +902,7 @@
       <c r="K14" t="inlineStr"/>
       <c r="L14" t="inlineStr">
         <is>
-          <t>E:\geology\(2012)_Carbonates.pdf</t>
+          <t>E:\todos os textos\(1955)_Homogeny.pdf</t>
         </is>
       </c>
       <c r="M14" t="inlineStr"/>
@@ -913,11 +913,11 @@
       </c>
       <c r="O14" t="inlineStr">
         <is>
-          <t>replacement of bioclasts by a mixture of dolomite and homogeneous textures in breccia facies of the waulsortian mound</t>
+          <t>aping of a modem language extent to which a homogeneous texture a texture in which all the parts share the same</t>
         </is>
       </c>
       <c r="P14" t="n">
-        <v>18</v>
+        <v>21</v>
       </c>
     </row>
     <row r="15">
@@ -928,7 +928,7 @@
       <c r="E15" t="inlineStr"/>
       <c r="F15" t="inlineStr">
         <is>
-          <t>textura</t>
+          <t>textures</t>
         </is>
       </c>
       <c r="G15" t="inlineStr"/>
@@ -938,7 +938,7 @@
       <c r="K15" t="inlineStr"/>
       <c r="L15" t="inlineStr">
         <is>
-          <t>E:\todos os textos\(2010)_Textura_PT.pdf</t>
+          <t>E:\geology\(2012)_Carbonates.pdf</t>
         </is>
       </c>
       <c r="M15" t="inlineStr"/>
@@ -949,11 +949,11 @@
       </c>
       <c r="O15" t="inlineStr">
         <is>
-          <t>a obra apresenta uma textura homogenea de cordas no andante e um contraste timbrico no finale</t>
+          <t>replacement of bioclasts by a mixture of dolomite and homogeneous textures in breccia facies of the waulsortian mound</t>
         </is>
       </c>
       <c r="P15" t="n">
-        <v>16</v>
+        <v>18</v>
       </c>
     </row>
     <row r="16">
@@ -974,7 +974,7 @@
       <c r="K16" t="inlineStr"/>
       <c r="L16" t="inlineStr">
         <is>
-          <t>E:\todos os textos\(2011)_Coral_PT.pdf</t>
+          <t>E:\todos os textos\(2010)_Textura_PT.pdf</t>
         </is>
       </c>
       <c r="M16" t="inlineStr"/>
@@ -985,11 +985,11 @@
       </c>
       <c r="O16" t="inlineStr">
         <is>
-          <t>nao se observa uma textura uniforme no coral apesar da escrita a quatro vozes</t>
+          <t>a obra apresenta uma textura homogenea de cordas no andante e um contraste timbrico no finale</t>
         </is>
       </c>
       <c r="P16" t="n">
-        <v>14</v>
+        <v>16</v>
       </c>
     </row>
     <row r="17">
@@ -1000,7 +1000,7 @@
       <c r="E17" t="inlineStr"/>
       <c r="F17" t="inlineStr">
         <is>
-          <t>texturas</t>
+          <t>textura</t>
         </is>
       </c>
       <c r="G17" t="inlineStr"/>
@@ -1010,7 +1010,7 @@
       <c r="K17" t="inlineStr"/>
       <c r="L17" t="inlineStr">
         <is>
-          <t>E:\todos os textos\(2014)_Acomp_PT.pdf</t>
+          <t>E:\todos os textos\(2011)_Coral_PT.pdf</t>
         </is>
       </c>
       <c r="M17" t="inlineStr"/>
@@ -1021,11 +1021,11 @@
       </c>
       <c r="O17" t="inlineStr">
         <is>
-          <t>as texturas constantes do acompanhamento sustentam a melodia principal sem variar o ritmo</t>
+          <t>nao se observa uma textura uniforme no coral apesar da escrita a quatro vozes</t>
         </is>
       </c>
       <c r="P17" t="n">
-        <v>13</v>
+        <v>14</v>
       </c>
     </row>
     <row r="18">
@@ -1036,7 +1036,7 @@
       <c r="E18" t="inlineStr"/>
       <c r="F18" t="inlineStr">
         <is>
-          <t>texture</t>
+          <t>texturas</t>
         </is>
       </c>
       <c r="G18" t="inlineStr"/>
@@ -1046,7 +1046,7 @@
       <c r="K18" t="inlineStr"/>
       <c r="L18" t="inlineStr">
         <is>
-          <t>E:\todos os textos\(1975)_Woodwind.pdf</t>
+          <t>E:\todos os textos\(2014)_Acomp_PT.pdf</t>
         </is>
       </c>
       <c r="M18" t="inlineStr"/>
@@ -1057,11 +1057,11 @@
       </c>
       <c r="O18" t="inlineStr">
         <is>
-          <t>a stable texture of woodwind chords supports the solo line in the slow movement</t>
+          <t>as texturas constantes do acompanhamento sustentam a melodia principal sem variar o ritmo</t>
         </is>
       </c>
       <c r="P18" t="n">
-        <v>14</v>
+        <v>13</v>
       </c>
     </row>
     <row r="19">
@@ -1082,7 +1082,7 @@
       <c r="K19" t="inlineStr"/>
       <c r="L19" t="inlineStr">
         <is>
-          <t>E:\todos os textos\(1977)_Scherzo.pdf</t>
+          <t>E:\todos os textos\(1975)_Woodwind.pdf</t>
         </is>
       </c>
       <c r="M19" t="inlineStr"/>
@@ -1093,7 +1093,7 @@
       </c>
       <c r="O19" t="inlineStr">
         <is>
-          <t>the varied texture of the scherzo contrasts with the sustained chords of the trio</t>
+          <t>a stable texture of woodwind chords supports the solo line in the slow movement</t>
         </is>
       </c>
       <c r="P19" t="n">
@@ -1118,7 +1118,7 @@
       <c r="K20" t="inlineStr"/>
       <c r="L20" t="inlineStr">
         <is>
-          <t>E:\todos os textos\(1982)_Pizz.pdf</t>
+          <t>E:\todos os textos\(1977)_Scherzo.pdf</t>
         </is>
       </c>
       <c r="M20" t="inlineStr"/>
@@ -1129,11 +1129,11 @@
       </c>
       <c r="O20" t="inlineStr">
         <is>
-          <t>an irregular texture of pizzicato fragments interrupts the otherwise calm surface</t>
+          <t>the varied texture of the scherzo contrasts with the sustained chords of the trio</t>
         </is>
       </c>
       <c r="P20" t="n">
-        <v>11</v>
+        <v>14</v>
       </c>
     </row>
     <row r="21">
@@ -1144,7 +1144,7 @@
       <c r="E21" t="inlineStr"/>
       <c r="F21" t="inlineStr">
         <is>
-          <t>textural</t>
+          <t>texture</t>
         </is>
       </c>
       <c r="G21" t="inlineStr"/>
@@ -1154,7 +1154,7 @@
       <c r="K21" t="inlineStr"/>
       <c r="L21" t="inlineStr">
         <is>
-          <t>E:\todos os textos\(1988)_Density.pdf</t>
+          <t>E:\todos os textos\(1982)_Pizz.pdf</t>
         </is>
       </c>
       <c r="M21" t="inlineStr"/>
@@ -1165,11 +1165,11 @@
       </c>
       <c r="O21" t="inlineStr">
         <is>
-          <t>textural density increases as the consistent pulse of the ostinato thickens the fabric</t>
+          <t>an irregular texture of pizzicato fragments interrupts the otherwise calm surface</t>
         </is>
       </c>
       <c r="P21" t="n">
-        <v>13</v>
+        <v>11</v>
       </c>
     </row>
     <row r="22">
@@ -1180,7 +1180,7 @@
       <c r="E22" t="inlineStr"/>
       <c r="F22" t="inlineStr">
         <is>
-          <t>texture</t>
+          <t>textural</t>
         </is>
       </c>
       <c r="G22" t="inlineStr"/>
@@ -1190,7 +1190,7 @@
       <c r="K22" t="inlineStr"/>
       <c r="L22" t="inlineStr">
         <is>
-          <t>E:\todos os textos\(1992)_Static.pdf</t>
+          <t>E:\todos os textos\(1988)_Density.pdf</t>
         </is>
       </c>
       <c r="M22" t="inlineStr"/>
@@ -1201,11 +1201,11 @@
       </c>
       <c r="O22" t="inlineStr">
         <is>
-          <t>the static texture of the opening is soon abandoned for a changing web of lines</t>
+          <t>textural density increases as the consistent pulse of the ostinato thickens the fabric</t>
         </is>
       </c>
       <c r="P22" t="n">
-        <v>15</v>
+        <v>13</v>
       </c>
     </row>
     <row r="23">
@@ -1226,7 +1226,7 @@
       <c r="K23" t="inlineStr"/>
       <c r="L23" t="inlineStr">
         <is>
-          <t>E:\todos os textos\(1995)_Adagio.pdf</t>
+          <t>E:\todos os textos\(1992)_Static.pdf</t>
         </is>
       </c>
       <c r="M23" t="inlineStr"/>
@@ -1237,11 +1237,11 @@
       </c>
       <c r="O23" t="inlineStr">
         <is>
-          <t>critics praised the sustained texture of the adagio as a model of orchestral balance</t>
+          <t>the static texture of the opening is soon abandoned for a changing web of lines</t>
         </is>
       </c>
       <c r="P23" t="n">
-        <v>14</v>
+        <v>15</v>
       </c>
     </row>
     <row r="24">
@@ -1262,7 +1262,7 @@
       <c r="K24" t="inlineStr"/>
       <c r="L24" t="inlineStr">
         <is>
-          <t>E:\todos os textos\(1998)_Dance.pdf</t>
+          <t>E:\todos os textos\(1995)_Adagio.pdf</t>
         </is>
       </c>
       <c r="M24" t="inlineStr"/>
@@ -1273,11 +1273,11 @@
       </c>
       <c r="O24" t="inlineStr">
         <is>
-          <t>a regular texture of repeated chords marks the dance refrain of the suite</t>
+          <t>critics praised the sustained texture of the adagio as a model of orchestral balance</t>
         </is>
       </c>
       <c r="P24" t="n">
-        <v>13</v>
+        <v>14</v>
       </c>
     </row>
     <row r="25">
@@ -1298,7 +1298,7 @@
       <c r="K25" t="inlineStr"/>
       <c r="L25" t="inlineStr">
         <is>
-          <t>E:\todos os textos\(2003)_Drone.pdf</t>
+          <t>E:\todos os textos\(1998)_Dance.pdf</t>
         </is>
       </c>
       <c r="M25" t="inlineStr"/>
@@ -1309,11 +1309,11 @@
       </c>
       <c r="O25" t="inlineStr">
         <is>
-          <t>the immutable texture of the drone underpins the improvisation of the soloist</t>
+          <t>a regular texture of repeated chords marks the dance refrain of the suite</t>
         </is>
       </c>
       <c r="P25" t="n">
-        <v>12</v>
+        <v>13</v>
       </c>
     </row>
     <row r="26">
@@ -1334,7 +1334,7 @@
       <c r="K26" t="inlineStr"/>
       <c r="L26" t="inlineStr">
         <is>
-          <t>E:\todos os textos\(2006)_Narration.pdf</t>
+          <t>E:\todos os textos\(2003)_Drone.pdf</t>
         </is>
       </c>
       <c r="M26" t="inlineStr"/>
@@ -1345,11 +1345,11 @@
       </c>
       <c r="O26" t="inlineStr">
         <is>
-          <t>an unchanging texture of muted strings accompanies the spoken narration throughout</t>
+          <t>the immutable texture of the drone underpins the improvisation of the soloist</t>
         </is>
       </c>
       <c r="P26" t="n">
-        <v>11</v>
+        <v>12</v>
       </c>
     </row>
     <row r="27">
@@ -1370,7 +1370,7 @@
       <c r="K27" t="inlineStr"/>
       <c r="L27" t="inlineStr">
         <is>
-          <t>E:\todos os textos\(2009)_March.pdf</t>
+          <t>E:\todos os textos\(2006)_Narration.pdf</t>
         </is>
       </c>
       <c r="M27" t="inlineStr"/>
@@ -1381,10 +1381,46 @@
       </c>
       <c r="O27" t="inlineStr">
         <is>
+          <t>an unchanging texture of muted strings accompanies the spoken narration throughout</t>
+        </is>
+      </c>
+      <c r="P27" t="n">
+        <v>11</v>
+      </c>
+    </row>
+    <row r="28">
+      <c r="A28" t="inlineStr"/>
+      <c r="B28" t="inlineStr"/>
+      <c r="C28" t="inlineStr"/>
+      <c r="D28" t="inlineStr"/>
+      <c r="E28" t="inlineStr"/>
+      <c r="F28" t="inlineStr">
+        <is>
+          <t>texture</t>
+        </is>
+      </c>
+      <c r="G28" t="inlineStr"/>
+      <c r="H28" t="inlineStr"/>
+      <c r="I28" t="inlineStr"/>
+      <c r="J28" t="inlineStr"/>
+      <c r="K28" t="inlineStr"/>
+      <c r="L28" t="inlineStr">
+        <is>
+          <t>E:\todos os textos\(2009)_March.pdf</t>
+        </is>
+      </c>
+      <c r="M28" t="inlineStr"/>
+      <c r="N28" t="inlineStr">
+        <is>
+          <t>raiz</t>
+        </is>
+      </c>
+      <c r="O28" t="inlineStr">
+        <is>
           <t>a constant texture of muted brass underpins the funeral march of the symphony</t>
         </is>
       </c>
-      <c r="P27" t="n">
+      <c r="P28" t="n">
         <v>13</v>
       </c>
     </row>

</xml_diff>

<commit_message>
Add FR golden path and enrich PT; restore strict ruff F401.
FR is first-class for dissertation counts (pinned fr_core_news_sm + thin golden); PT gains genitive/coordination locks; EN golden uses --lingua en; shim re-exports declared so F401 stays global.

Co-authored-by: Cursor <cursoragent@cursor.com>
</commit_message>
<xml_diff>
--- a/tests/fixtures/matriz_miniatura.xlsx
+++ b/tests/fixtures/matriz_miniatura.xlsx
@@ -413,7 +413,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:P28"/>
+  <dimension ref="A1:P31"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -1072,7 +1072,7 @@
       <c r="E19" t="inlineStr"/>
       <c r="F19" t="inlineStr">
         <is>
-          <t>texture</t>
+          <t>textura</t>
         </is>
       </c>
       <c r="G19" t="inlineStr"/>
@@ -1082,7 +1082,7 @@
       <c r="K19" t="inlineStr"/>
       <c r="L19" t="inlineStr">
         <is>
-          <t>E:\todos os textos\(1975)_Woodwind.pdf</t>
+          <t>E:\todos os textos\(2012)_Complexidade_PT.pdf</t>
         </is>
       </c>
       <c r="M19" t="inlineStr"/>
@@ -1093,11 +1093,11 @@
       </c>
       <c r="O19" t="inlineStr">
         <is>
-          <t>a stable texture of woodwind chords supports the solo line in the slow movement</t>
+          <t>a complexidade da textura caracteriza o segundo tema do allegro</t>
         </is>
       </c>
       <c r="P19" t="n">
-        <v>14</v>
+        <v>10</v>
       </c>
     </row>
     <row r="20">
@@ -1108,7 +1108,7 @@
       <c r="E20" t="inlineStr"/>
       <c r="F20" t="inlineStr">
         <is>
-          <t>texture</t>
+          <t>textura</t>
         </is>
       </c>
       <c r="G20" t="inlineStr"/>
@@ -1118,7 +1118,7 @@
       <c r="K20" t="inlineStr"/>
       <c r="L20" t="inlineStr">
         <is>
-          <t>E:\todos os textos\(1977)_Scherzo.pdf</t>
+          <t>E:\todos os textos\(2013)_Combinacao_PT.pdf</t>
         </is>
       </c>
       <c r="M20" t="inlineStr"/>
@@ -1129,11 +1129,11 @@
       </c>
       <c r="O20" t="inlineStr">
         <is>
-          <t>the varied texture of the scherzo contrasts with the sustained chords of the trio</t>
+          <t>a textura complexa e a dinamica contrastante no coral final</t>
         </is>
       </c>
       <c r="P20" t="n">
-        <v>14</v>
+        <v>10</v>
       </c>
     </row>
     <row r="21">
@@ -1144,7 +1144,7 @@
       <c r="E21" t="inlineStr"/>
       <c r="F21" t="inlineStr">
         <is>
-          <t>texture</t>
+          <t>textura</t>
         </is>
       </c>
       <c r="G21" t="inlineStr"/>
@@ -1154,7 +1154,7 @@
       <c r="K21" t="inlineStr"/>
       <c r="L21" t="inlineStr">
         <is>
-          <t>E:\todos os textos\(1982)_Pizz.pdf</t>
+          <t>E:\todos os textos\(2015)_Negacao_PT.pdf</t>
         </is>
       </c>
       <c r="M21" t="inlineStr"/>
@@ -1165,11 +1165,11 @@
       </c>
       <c r="O21" t="inlineStr">
         <is>
-          <t>an irregular texture of pizzicato fragments interrupts the otherwise calm surface</t>
+          <t>a passagem nao apresenta textura uniforme no coral final</t>
         </is>
       </c>
       <c r="P21" t="n">
-        <v>11</v>
+        <v>9</v>
       </c>
     </row>
     <row r="22">
@@ -1180,7 +1180,7 @@
       <c r="E22" t="inlineStr"/>
       <c r="F22" t="inlineStr">
         <is>
-          <t>textural</t>
+          <t>texture</t>
         </is>
       </c>
       <c r="G22" t="inlineStr"/>
@@ -1190,7 +1190,7 @@
       <c r="K22" t="inlineStr"/>
       <c r="L22" t="inlineStr">
         <is>
-          <t>E:\todos os textos\(1988)_Density.pdf</t>
+          <t>E:\todos os textos\(1975)_Woodwind.pdf</t>
         </is>
       </c>
       <c r="M22" t="inlineStr"/>
@@ -1201,11 +1201,11 @@
       </c>
       <c r="O22" t="inlineStr">
         <is>
-          <t>textural density increases as the consistent pulse of the ostinato thickens the fabric</t>
+          <t>a stable texture of woodwind chords supports the solo line in the slow movement</t>
         </is>
       </c>
       <c r="P22" t="n">
-        <v>13</v>
+        <v>14</v>
       </c>
     </row>
     <row r="23">
@@ -1226,7 +1226,7 @@
       <c r="K23" t="inlineStr"/>
       <c r="L23" t="inlineStr">
         <is>
-          <t>E:\todos os textos\(1992)_Static.pdf</t>
+          <t>E:\todos os textos\(1977)_Scherzo.pdf</t>
         </is>
       </c>
       <c r="M23" t="inlineStr"/>
@@ -1237,11 +1237,11 @@
       </c>
       <c r="O23" t="inlineStr">
         <is>
-          <t>the static texture of the opening is soon abandoned for a changing web of lines</t>
+          <t>the varied texture of the scherzo contrasts with the sustained chords of the trio</t>
         </is>
       </c>
       <c r="P23" t="n">
-        <v>15</v>
+        <v>14</v>
       </c>
     </row>
     <row r="24">
@@ -1262,7 +1262,7 @@
       <c r="K24" t="inlineStr"/>
       <c r="L24" t="inlineStr">
         <is>
-          <t>E:\todos os textos\(1995)_Adagio.pdf</t>
+          <t>E:\todos os textos\(1982)_Pizz.pdf</t>
         </is>
       </c>
       <c r="M24" t="inlineStr"/>
@@ -1273,11 +1273,11 @@
       </c>
       <c r="O24" t="inlineStr">
         <is>
-          <t>critics praised the sustained texture of the adagio as a model of orchestral balance</t>
+          <t>an irregular texture of pizzicato fragments interrupts the otherwise calm surface</t>
         </is>
       </c>
       <c r="P24" t="n">
-        <v>14</v>
+        <v>11</v>
       </c>
     </row>
     <row r="25">
@@ -1288,7 +1288,7 @@
       <c r="E25" t="inlineStr"/>
       <c r="F25" t="inlineStr">
         <is>
-          <t>texture</t>
+          <t>textural</t>
         </is>
       </c>
       <c r="G25" t="inlineStr"/>
@@ -1298,7 +1298,7 @@
       <c r="K25" t="inlineStr"/>
       <c r="L25" t="inlineStr">
         <is>
-          <t>E:\todos os textos\(1998)_Dance.pdf</t>
+          <t>E:\todos os textos\(1988)_Density.pdf</t>
         </is>
       </c>
       <c r="M25" t="inlineStr"/>
@@ -1309,7 +1309,7 @@
       </c>
       <c r="O25" t="inlineStr">
         <is>
-          <t>a regular texture of repeated chords marks the dance refrain of the suite</t>
+          <t>textural density increases as the consistent pulse of the ostinato thickens the fabric</t>
         </is>
       </c>
       <c r="P25" t="n">
@@ -1334,7 +1334,7 @@
       <c r="K26" t="inlineStr"/>
       <c r="L26" t="inlineStr">
         <is>
-          <t>E:\todos os textos\(2003)_Drone.pdf</t>
+          <t>E:\todos os textos\(1992)_Static.pdf</t>
         </is>
       </c>
       <c r="M26" t="inlineStr"/>
@@ -1345,11 +1345,11 @@
       </c>
       <c r="O26" t="inlineStr">
         <is>
-          <t>the immutable texture of the drone underpins the improvisation of the soloist</t>
+          <t>the static texture of the opening is soon abandoned for a changing web of lines</t>
         </is>
       </c>
       <c r="P26" t="n">
-        <v>12</v>
+        <v>15</v>
       </c>
     </row>
     <row r="27">
@@ -1370,7 +1370,7 @@
       <c r="K27" t="inlineStr"/>
       <c r="L27" t="inlineStr">
         <is>
-          <t>E:\todos os textos\(2006)_Narration.pdf</t>
+          <t>E:\todos os textos\(1995)_Adagio.pdf</t>
         </is>
       </c>
       <c r="M27" t="inlineStr"/>
@@ -1381,11 +1381,11 @@
       </c>
       <c r="O27" t="inlineStr">
         <is>
-          <t>an unchanging texture of muted strings accompanies the spoken narration throughout</t>
+          <t>critics praised the sustained texture of the adagio as a model of orchestral balance</t>
         </is>
       </c>
       <c r="P27" t="n">
-        <v>11</v>
+        <v>14</v>
       </c>
     </row>
     <row r="28">
@@ -1406,7 +1406,7 @@
       <c r="K28" t="inlineStr"/>
       <c r="L28" t="inlineStr">
         <is>
-          <t>E:\todos os textos\(2009)_March.pdf</t>
+          <t>E:\todos os textos\(1998)_Dance.pdf</t>
         </is>
       </c>
       <c r="M28" t="inlineStr"/>
@@ -1417,10 +1417,118 @@
       </c>
       <c r="O28" t="inlineStr">
         <is>
+          <t>a regular texture of repeated chords marks the dance refrain of the suite</t>
+        </is>
+      </c>
+      <c r="P28" t="n">
+        <v>13</v>
+      </c>
+    </row>
+    <row r="29">
+      <c r="A29" t="inlineStr"/>
+      <c r="B29" t="inlineStr"/>
+      <c r="C29" t="inlineStr"/>
+      <c r="D29" t="inlineStr"/>
+      <c r="E29" t="inlineStr"/>
+      <c r="F29" t="inlineStr">
+        <is>
+          <t>texture</t>
+        </is>
+      </c>
+      <c r="G29" t="inlineStr"/>
+      <c r="H29" t="inlineStr"/>
+      <c r="I29" t="inlineStr"/>
+      <c r="J29" t="inlineStr"/>
+      <c r="K29" t="inlineStr"/>
+      <c r="L29" t="inlineStr">
+        <is>
+          <t>E:\todos os textos\(2003)_Drone.pdf</t>
+        </is>
+      </c>
+      <c r="M29" t="inlineStr"/>
+      <c r="N29" t="inlineStr">
+        <is>
+          <t>raiz</t>
+        </is>
+      </c>
+      <c r="O29" t="inlineStr">
+        <is>
+          <t>the immutable texture of the drone underpins the improvisation of the soloist</t>
+        </is>
+      </c>
+      <c r="P29" t="n">
+        <v>12</v>
+      </c>
+    </row>
+    <row r="30">
+      <c r="A30" t="inlineStr"/>
+      <c r="B30" t="inlineStr"/>
+      <c r="C30" t="inlineStr"/>
+      <c r="D30" t="inlineStr"/>
+      <c r="E30" t="inlineStr"/>
+      <c r="F30" t="inlineStr">
+        <is>
+          <t>texture</t>
+        </is>
+      </c>
+      <c r="G30" t="inlineStr"/>
+      <c r="H30" t="inlineStr"/>
+      <c r="I30" t="inlineStr"/>
+      <c r="J30" t="inlineStr"/>
+      <c r="K30" t="inlineStr"/>
+      <c r="L30" t="inlineStr">
+        <is>
+          <t>E:\todos os textos\(2006)_Narration.pdf</t>
+        </is>
+      </c>
+      <c r="M30" t="inlineStr"/>
+      <c r="N30" t="inlineStr">
+        <is>
+          <t>raiz</t>
+        </is>
+      </c>
+      <c r="O30" t="inlineStr">
+        <is>
+          <t>an unchanging texture of muted strings accompanies the spoken narration throughout</t>
+        </is>
+      </c>
+      <c r="P30" t="n">
+        <v>11</v>
+      </c>
+    </row>
+    <row r="31">
+      <c r="A31" t="inlineStr"/>
+      <c r="B31" t="inlineStr"/>
+      <c r="C31" t="inlineStr"/>
+      <c r="D31" t="inlineStr"/>
+      <c r="E31" t="inlineStr"/>
+      <c r="F31" t="inlineStr">
+        <is>
+          <t>texture</t>
+        </is>
+      </c>
+      <c r="G31" t="inlineStr"/>
+      <c r="H31" t="inlineStr"/>
+      <c r="I31" t="inlineStr"/>
+      <c r="J31" t="inlineStr"/>
+      <c r="K31" t="inlineStr"/>
+      <c r="L31" t="inlineStr">
+        <is>
+          <t>E:\todos os textos\(2009)_March.pdf</t>
+        </is>
+      </c>
+      <c r="M31" t="inlineStr"/>
+      <c r="N31" t="inlineStr">
+        <is>
+          <t>raiz</t>
+        </is>
+      </c>
+      <c r="O31" t="inlineStr">
+        <is>
           <t>a constant texture of muted brass underpins the funeral march of the symphony</t>
         </is>
       </c>
-      <c r="P28" t="n">
+      <c r="P31" t="n">
         <v>13</v>
       </c>
     </row>

</xml_diff>